<commit_message>
docs(B-L1): reconcile privacy policy + mark B-L1 done in checklist/tracker
Privacy policy (docs/privacy/index.html) updated to match Option A: removed Google Vision + Anthropic
third parties, added explicit 'never sent to any AI/LLM provider' + on-device tips/OCR. Checklist B-L1
→ done (re-host policy remains 🧑); Excel + flat tracker updated (open blockers 20 → 19).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/finwise-launch-checklist.xlsx
+++ b/docs/finwise-launch-checklist.xlsx
@@ -401,15 +401,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G39"/>
-  <cols>
-    <col min="1" max="1" width="30.83203125" customWidth="1"/>
-    <col min="2" max="2" width="7.83203125" customWidth="1"/>
-    <col min="3" max="3" width="62.83203125" customWidth="1"/>
-    <col min="4" max="4" width="8.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="55.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -957,10 +948,10 @@
         <v>Blocker</v>
       </c>
       <c r="F24" t="str">
-        <v>Open</v>
+        <v>Done</v>
       </c>
       <c r="G24" t="str">
-        <v>Ship AI-tips off OR add consent+disclosure+policy; scope claim to "stored data"</v>
+        <v>DONE 945f929 — on-device tips + OCR; claim updated; policy reconciled; re-host policy = 🧑</v>
       </c>
     </row>
     <row r="25">

</xml_diff>

<commit_message>
docs: mark B-L3 + B-L4 done in checklist/tracker (open blockers 19 → 17)
</commit_message>
<xml_diff>
--- a/docs/finwise-launch-checklist.xlsx
+++ b/docs/finwise-launch-checklist.xlsx
@@ -994,10 +994,10 @@
         <v>Blocker</v>
       </c>
       <c r="F26" t="str">
-        <v>Open</v>
+        <v>Done</v>
       </c>
       <c r="G26" t="str">
-        <v>Verified by test/screenshot pass</v>
+        <v>DONE bb68bad — shared &lt;Disclaimer/&gt; on all 5 judgment screens; RMD phrased as IRS requirement; guard test</v>
       </c>
     </row>
     <row r="27">
@@ -1017,10 +1017,10 @@
         <v>Blocker</v>
       </c>
       <c r="F27" t="str">
-        <v>Open</v>
+        <v>Done</v>
       </c>
       <c r="G27" t="str">
-        <v>No thrown error / corrupted projection on failure; test</v>
+        <v>DONE (verified) — all wired network paths already degrade gracefully (prices allSettled+null keep-cache; econ allSettled+fallback flags; econ feed unwired, inflation static default). Covered by existing tests; no code change.</v>
       </c>
     </row>
     <row r="28">

</xml_diff>

<commit_message>
docs(R-1/R-3/R-2): ledger verified clean, App Review note drafted, Maestro runbook ready
R-1: bug ledger verified — all 42 rows fixed, 0 open, no user-facing money error; corrected the stale
summary header. R-3: docs/finwise-app-review-notes.md drafted (educational-tool framing to de-risk the
fintech-licensing guideline + reviewer demo-login placeholder + recovery-code walkthrough). R-2: the
on-device Maestro runbook already covers all 5 flows (.maestro/README) — ready for the user to run.
Tracker updated.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/finwise-launch-checklist.xlsx
+++ b/docs/finwise-launch-checklist.xlsx
@@ -1040,10 +1040,10 @@
         <v>Important</v>
       </c>
       <c r="F28" t="str">
-        <v>Open</v>
+        <v>Done</v>
       </c>
       <c r="G28" t="str">
-        <v>docs/finwise-bug-ledger.md</v>
+        <v>VERIFIED — ledger 0 open; all 42 fixed; stale summary header corrected (no money error open)</v>
       </c>
     </row>
     <row r="29">
@@ -1063,10 +1063,10 @@
         <v>Important</v>
       </c>
       <c r="F29" t="str">
-        <v>Open</v>
+        <v>Ready</v>
       </c>
       <c r="G29" t="str">
-        <v>auth-signup, smoke, b21-add-sheet, nw-donut, cashflow</v>
+        <v>RUNBOOK ready in .maestro/README (npm run test:e2e, 5 flows); 🧑 runs on a real device</v>
       </c>
     </row>
     <row r="30">
@@ -1086,10 +1086,10 @@
         <v>Important</v>
       </c>
       <c r="F30" t="str">
-        <v>Open</v>
+        <v>Done</v>
       </c>
       <c r="G30" t="str">
-        <v>De-risks fintech-licensing guideline</v>
+        <v>DRAFTED — docs/finwise-app-review-notes.md (educational-tool note + demo-login placeholder); 🧑 fill creds + paste</v>
       </c>
     </row>
     <row r="31">

</xml_diff>

<commit_message>
docs: B-L2 code pre-staged — tracker/checklist updated (awaiting Sentry DSN)
</commit_message>
<xml_diff>
--- a/docs/finwise-launch-checklist.xlsx
+++ b/docs/finwise-launch-checklist.xlsx
@@ -971,10 +971,10 @@
         <v>Blocker</v>
       </c>
       <c r="F25" t="str">
-        <v>Open</v>
+        <v>Code ready</v>
       </c>
       <c r="G25" t="str">
-        <v>Forced test crash appears in dashboard</v>
+        <v>PRE-STAGED f43819e — DSN-ready, latent report bug fixed, test-report row + policy. 🧑: Sentry project + DSN + install + rebuild (docs/finwise-sentry-setup.md). Verify event in dashboard.</v>
       </c>
     </row>
     <row r="26">

</xml_diff>

<commit_message>
docs: B-L2 wired (org/project/DSN/plugin/metro) — verify in next build
</commit_message>
<xml_diff>
--- a/docs/finwise-launch-checklist.xlsx
+++ b/docs/finwise-launch-checklist.xlsx
@@ -971,10 +971,10 @@
         <v>Blocker</v>
       </c>
       <c r="F25" t="str">
-        <v>Code ready</v>
+        <v>Wired</v>
       </c>
       <c r="G25" t="str">
-        <v>PRE-STAGED f43819e — DSN-ready, latent report bug fixed, test-report row + policy. 🧑: Sentry project + DSN + install + rebuild (docs/finwise-sentry-setup.md). Verify event in dashboard.</v>
+        <v>WIRED 3937f04 — DSN+Expo plugin(org finwise-35/proj react-native)+Metro source maps+loader. Live in next build. DONE when test event shows in dashboard (Settings -&gt; Send a diagnostic report).</v>
       </c>
     </row>
     <row r="26">

</xml_diff>

<commit_message>
docs: add A-1/A-2 accuracy P0s to launch checklist (a wrong number = lost trust)
A-1: %-of-income base for % spending categories differs between screen and domain budget. A-2:
systematic cross-screen money-agreement audit — every displayed money concept single-sourced + pinned
by a test asserting the rendered number matches on every screen (accuracy checkable, not trusted).
Two such bugs already found (#6, B-67) → class not closed.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/finwise-launch-checklist.xlsx
+++ b/docs/finwise-launch-checklist.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Launch Checklist" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Launch Checklist'!A1:G39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Launch Checklist'!A1:G41</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G41"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -971,10 +971,10 @@
         <v>Blocker</v>
       </c>
       <c r="F25" t="str">
-        <v>Wired</v>
+        <v>Code ready</v>
       </c>
       <c r="G25" t="str">
-        <v>WIRED 3937f04 — DSN+Expo plugin(org finwise-35/proj react-native)+Metro source maps+loader. Live in next build. DONE when test event shows in dashboard (Settings -&gt; Send a diagnostic report).</v>
+        <v>PRE-STAGED f43819e — DSN-ready, latent report bug fixed, test-report row + policy. 🧑: Sentry project + DSN + install + rebuild (docs/finwise-sentry-setup.md). Verify event in dashboard.</v>
       </c>
     </row>
     <row r="26">
@@ -1140,94 +1140,94 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Phase 3 — Optional (post-v1)</v>
+        <v>Phase 2.6 — Launch-review findings</v>
       </c>
       <c r="B33" t="str">
-        <v>P3.1</v>
+        <v>A-1</v>
       </c>
       <c r="C33" t="str">
-        <v>Plaid bank linking</v>
+        <v>%-of-income base for % spending categories differs between the spending screen and the domain budget (net-of-tax vs take-home) — screen $ ≠ budget $</v>
       </c>
       <c r="D33" t="str">
-        <v>🧑</v>
+        <v>🤖</v>
       </c>
       <c r="E33" t="str">
-        <v>Optional</v>
+        <v>Blocker</v>
       </c>
       <c r="F33" t="str">
         <v>Open</v>
       </c>
       <c r="G33" t="str">
-        <v>Needs Plaid keys + backend</v>
+        <v>One income base (take-home, after tax+401k) for every %-category conversion; test: screen-displayed $ == domain $ for a % category (incl 401k); golden reconciled</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Phase 3 — Optional (post-v1)</v>
+        <v>Phase 2.6 — Launch-review findings</v>
       </c>
       <c r="B34" t="str">
-        <v>P3.2</v>
+        <v>A-2</v>
       </c>
       <c r="C34" t="str">
-        <v>Push notifications</v>
+        <v>Systematic cross-screen money-agreement audit: every displayed money concept single-sourced + pinned by a test asserting the rendered number is identical on every screen</v>
       </c>
       <c r="D34" t="str">
-        <v>🧑</v>
+        <v>🤖</v>
       </c>
       <c r="E34" t="str">
-        <v>Optional</v>
+        <v>Blocker</v>
       </c>
       <c r="F34" t="str">
         <v>Open</v>
       </c>
       <c r="G34" t="str">
-        <v>Needs APNs + reminder logic</v>
+        <v>Traceability matrix concept→helper→screens→test, green per row (accuracy checkable not trusted). L-7. Two already found: #6, B-67</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Phase 4 — Final pre-submit QA</v>
+        <v>Phase 3 — Optional (post-v1)</v>
       </c>
       <c r="B35" t="str">
-        <v>4.1</v>
+        <v>P3.1</v>
       </c>
       <c r="C35" t="str">
-        <v>Clean onboarding for each persona (numbers reconcile)</v>
+        <v>Plaid bank linking</v>
       </c>
       <c r="D35" t="str">
         <v>🧑</v>
       </c>
       <c r="E35" t="str">
-        <v>Blocker</v>
+        <v>Optional</v>
       </c>
       <c r="F35" t="str">
         <v>Open</v>
       </c>
       <c r="G35" t="str">
-        <v>student / variable / professional / retiree</v>
+        <v>Needs Plaid keys + backend</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Phase 4 — Final pre-submit QA</v>
+        <v>Phase 3 — Optional (post-v1)</v>
       </c>
       <c r="B36" t="str">
-        <v>4.2</v>
+        <v>P3.2</v>
       </c>
       <c r="C36" t="str">
-        <v>Prices load from the LICENSED provider (not Yahoo)</v>
+        <v>Push notifications</v>
       </c>
       <c r="D36" t="str">
         <v>🧑</v>
       </c>
       <c r="E36" t="str">
-        <v>Blocker</v>
+        <v>Optional</v>
       </c>
       <c r="F36" t="str">
         <v>Open</v>
       </c>
       <c r="G36" t="str">
-        <v/>
+        <v>Needs APNs + reminder logic</v>
       </c>
     </row>
     <row r="37">
@@ -1235,10 +1235,10 @@
         <v>Phase 4 — Final pre-submit QA</v>
       </c>
       <c r="B37" t="str">
-        <v>4.3</v>
+        <v>4.1</v>
       </c>
       <c r="C37" t="str">
-        <v>Sign up → log out → recover account → log back in</v>
+        <v>Clean onboarding for each persona (numbers reconcile)</v>
       </c>
       <c r="D37" t="str">
         <v>🧑</v>
@@ -1250,7 +1250,7 @@
         <v>Open</v>
       </c>
       <c r="G37" t="str">
-        <v/>
+        <v>student / variable / professional / retiree</v>
       </c>
     </row>
     <row r="38">
@@ -1258,16 +1258,16 @@
         <v>Phase 4 — Final pre-submit QA</v>
       </c>
       <c r="B38" t="str">
-        <v>4.4</v>
+        <v>4.2</v>
       </c>
       <c r="C38" t="str">
-        <v>Test on a physical device (gestures, keyboard, safe-area, large text)</v>
+        <v>Prices load from the LICENSED provider (not Yahoo)</v>
       </c>
       <c r="D38" t="str">
         <v>🧑</v>
       </c>
       <c r="E38" t="str">
-        <v>Recommended</v>
+        <v>Blocker</v>
       </c>
       <c r="F38" t="str">
         <v>Open</v>
@@ -1281,10 +1281,10 @@
         <v>Phase 4 — Final pre-submit QA</v>
       </c>
       <c r="B39" t="str">
-        <v>4.5</v>
+        <v>4.3</v>
       </c>
       <c r="C39" t="str">
-        <v>eas submit → TestFlight → submit for review</v>
+        <v>Sign up → log out → recover account → log back in</v>
       </c>
       <c r="D39" t="str">
         <v>🧑</v>
@@ -1299,10 +1299,56 @@
         <v/>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>Phase 4 — Final pre-submit QA</v>
+      </c>
+      <c r="B40" t="str">
+        <v>4.4</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Test on a physical device (gestures, keyboard, safe-area, large text)</v>
+      </c>
+      <c r="D40" t="str">
+        <v>🧑</v>
+      </c>
+      <c r="E40" t="str">
+        <v>Recommended</v>
+      </c>
+      <c r="F40" t="str">
+        <v>Open</v>
+      </c>
+      <c r="G40" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>Phase 4 — Final pre-submit QA</v>
+      </c>
+      <c r="B41" t="str">
+        <v>4.5</v>
+      </c>
+      <c r="C41" t="str">
+        <v>eas submit → TestFlight → submit for review</v>
+      </c>
+      <c r="D41" t="str">
+        <v>🧑</v>
+      </c>
+      <c r="E41" t="str">
+        <v>Blocker</v>
+      </c>
+      <c r="F41" t="str">
+        <v>Open</v>
+      </c>
+      <c r="G41" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G39"/>
+  <autoFilter ref="A1:G41"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G39"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G41"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>